<commit_message>
Add Block 5 bill construction E2E tests
</commit_message>
<xml_diff>
--- a/docs/Nearz_E2E_Journey_Suite.xlsx
+++ b/docs/Nearz_E2E_Journey_Suite.xlsx
@@ -3306,10 +3306,14 @@
       </c>
       <c r="B52" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C52" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C52" s="43" t="inlineStr">
+        <is>
+          <t>baseline: service bill, cash, all 15 report figures</t>
+        </is>
+      </c>
       <c r="D52" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3355,10 +3359,14 @@
       </c>
       <c r="B53" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C53" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C53" s="43" t="inlineStr">
+        <is>
+          <t>the PERSISTED invoice reconciles: lines - discount = taxable, + tax + round_off = net, cgst+sgst = tax</t>
+        </is>
+      </c>
       <c r="D53" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3404,10 +3412,14 @@
       </c>
       <c r="B54" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C54" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C54" s="43" t="inlineStr">
+        <is>
+          <t>the PAYMENT record: amount_paid, amount_due 0, mode, billed_at, payment row</t>
+        </is>
+      </c>
       <c r="D54" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3453,10 +3465,14 @@
       </c>
       <c r="B55" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C55" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C55" s="43" t="inlineStr">
+        <is>
+          <t>service + product; service_total and product_total kept apart on the invoice</t>
+        </is>
+      </c>
       <c r="D55" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3502,10 +3518,14 @@
       </c>
       <c r="B56" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C56" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C56" s="43" t="inlineStr">
+        <is>
+          <t>three service lines, still ONE bill</t>
+        </is>
+      </c>
       <c r="D56" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3551,10 +3571,14 @@
       </c>
       <c r="B57" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C57" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C57" s="43" t="inlineStr">
+        <is>
+          <t>a 10% discount comes off BEFORE tax</t>
+        </is>
+      </c>
       <c r="D57" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3600,10 +3624,14 @@
       </c>
       <c r="B58" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C58" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C58" s="43" t="inlineStr">
+        <is>
+          <t>flat 250 discount - a separate code path from pct, they add</t>
+        </is>
+      </c>
       <c r="D58" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3649,10 +3677,14 @@
       </c>
       <c r="B59" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C59" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C59" s="43" t="inlineStr">
+        <is>
+          <t>GST 18% split into equal CGST/SGST halves</t>
+        </is>
+      </c>
       <c r="D59" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3698,10 +3730,14 @@
       </c>
       <c r="B60" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C60" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C60" s="43" t="inlineStr">
+        <is>
+          <t>per-bill gst_enabled=false; no salon setting touched</t>
+        </is>
+      </c>
       <c r="D60" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3747,10 +3783,14 @@
       </c>
       <c r="B61" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C61" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C61" s="43" t="inlineStr">
+        <is>
+          <t>tax INCLUSIVE: 1000 listed = 1000 charged, 152.54 backed out</t>
+        </is>
+      </c>
       <c r="D61" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3796,10 +3836,14 @@
       </c>
       <c r="B62" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C62" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C62" s="43" t="inlineStr">
+        <is>
+          <t>tax EXCLUSIVE: the same basket costs 180 more; asserted against 060</t>
+        </is>
+      </c>
       <c r="D62" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3845,10 +3889,14 @@
       </c>
       <c r="B63" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C63" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C63" s="43" t="inlineStr">
+        <is>
+          <t>discount and GST together, in the right order</t>
+        </is>
+      </c>
       <c r="D63" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3894,10 +3942,14 @@
       </c>
       <c r="B64" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C64" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C64" s="43" t="inlineStr">
+        <is>
+          <t>the compound basket - found the Profit round-off (gross_revenue 1079.60, not 1080)</t>
+        </is>
+      </c>
       <c r="D64" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3943,10 +3995,14 @@
       </c>
       <c r="B65" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C65" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C65" s="43" t="inlineStr">
+        <is>
+          <t>round-off ON: whole rupees, and gross_payable + round_off == net_payable</t>
+        </is>
+      </c>
       <c r="D65" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -3992,10 +4048,14 @@
       </c>
       <c r="B66" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C66" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C66" s="43" t="inlineStr">
+        <is>
+          <t>round-off OFF: flips the SALON-WIDE setting and restores it in a verified finally block</t>
+        </is>
+      </c>
       <c r="D66" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4041,10 +4101,14 @@
       </c>
       <c r="B67" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C67" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C67" s="43" t="inlineStr">
+        <is>
+          <t>cash settlement reaches Payments</t>
+        </is>
+      </c>
       <c r="D67" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4090,10 +4154,14 @@
       </c>
       <c r="B68" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C68" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C68" s="43" t="inlineStr">
+        <is>
+          <t>card settlement reaches the reports identically to cash</t>
+        </is>
+      </c>
       <c r="D68" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4139,10 +4207,14 @@
       </c>
       <c r="B69" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C69" s="43" t="n"/>
+          <t>PARKED</t>
+        </is>
+      </c>
+      <c r="C69" s="43" t="inlineStr">
+        <is>
+          <t>PARKED - a split payment is a partial payment, disabled in the frontend</t>
+        </is>
+      </c>
       <c r="D69" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4188,10 +4260,14 @@
       </c>
       <c r="B70" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C70" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C70" s="43" t="inlineStr">
+        <is>
+          <t>a second payment on a settled bill: the BILL is not double-collected</t>
+        </is>
+      </c>
       <c r="D70" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4237,10 +4313,14 @@
       </c>
       <c r="B71" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C71" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C71" s="43" t="inlineStr">
+        <is>
+          <t>the bill reads back with a complete payment history and an invoice number</t>
+        </is>
+      </c>
       <c r="D71" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4286,10 +4366,14 @@
       </c>
       <c r="B72" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C72" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C72" s="43" t="inlineStr">
+        <is>
+          <t>a DRAFT quotes the same total it later charges</t>
+        </is>
+      </c>
       <c r="D72" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4335,10 +4419,14 @@
       </c>
       <c r="B73" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C73" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C73" s="43" t="inlineStr">
+        <is>
+          <t>basket edited before payment; the reports use the FINAL basket</t>
+        </is>
+      </c>
       <c r="D73" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4384,10 +4472,14 @@
       </c>
       <c r="B74" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C74" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C74" s="43" t="inlineStr">
+        <is>
+          <t>duplicate payment request: the REPORTS are not double-collected</t>
+        </is>
+      </c>
       <c r="D74" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4433,10 +4525,14 @@
       </c>
       <c r="B75" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C75" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C75" s="43" t="inlineStr">
+        <is>
+          <t>wrong payment amount refused, bill uncorrupted and still settleable</t>
+        </is>
+      </c>
       <c r="D75" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -4482,10 +4578,14 @@
       </c>
       <c r="B76" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C76" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C76" s="43" t="inlineStr">
+        <is>
+          <t>one sale, all six reports reconcile (Sales = Profit + tax)</t>
+        </is>
+      </c>
       <c r="D76" s="44" t="inlineStr">
         <is>
           <t>3</t>
@@ -11035,13 +11135,13 @@
         <v>25</v>
       </c>
       <c r="E6" s="48" t="n">
+        <v>24</v>
+      </c>
+      <c r="F6" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="48" t="n">
         <v>0</v>
-      </c>
-      <c r="F6" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="48" t="n">
-        <v>25</v>
       </c>
       <c r="H6" s="48" t="n">
         <v>295</v>
@@ -11052,7 +11152,7 @@
       </c>
       <c r="J6" s="48" t="inlineStr">
         <is>
-          <t>to write</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -11322,7 +11422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="100" customWidth="1" style="28" min="1" max="1"/>
@@ -11502,30 +11602,58 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="28" t="inlineStr">
         <is>
           <t>30 Aug 2026 - Block 4 (build order) built: API-E2E-026..050, appointment lifecycle</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="28" t="inlineStr">
         <is>
           <t>22 passing, 2 parked (036/037 - reschedule is feature-flagged off on salon 4550), 1 deliberately failing (049 = D18).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="28" t="inlineStr">
         <is>
           <t>Found while building: D17 (reports cached 60s, no write invalidates - this also explains and closes the old Finding B) and D18 (bills never link to appointments, so booked customers count as walk-ins).</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="28" t="inlineStr">
         <is>
           <t>Every Reports.snapshot read now carries a unique _qa parameter to defeat that 60s cache. Blocks 1-3 had been racing it since they were written.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>4 Sep 2026 - Block 5 (build order) built: API-E2E-051..075, bill construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>24 passing, 1 parked (068 - split payment needs partial payment, off in the frontend).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>The automation now lives in Documents\nearz-api-tests. api-service holds no test code at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Block 5 corrected the Profit model: gross_revenue is net_payable MINUS tax (so a rounded bill keeps 40p less), and net_profit then deducts cost of goods sold. Both only show up on baskets with a product and a discount - which is why they survived 100 earlier tests.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Blocks 6-10 E2E journey tests and complete 200-journey suite
- Add Block 6 (API-E2E-126..150): staff, attendance, and commission journeys
- Add Block 7 (API-E2E-151..170): products, inventory, and stock journeys
- Add Block 8 (API-E2E-171..180): expenses and profit journeys
- Add Block 9 (API-E2E-181..185): dashboard reconciliation journeys
- Add Block 10 (API-E2E-186..200): composite mega-journeys
- Add VerifyDefectsTest on-demand defect audit suite
- Update Reports.java, Steps.java, testng.xml, README.md, DEFECTS.md, and test suite tracker
- Update .gitignore to exclude temporary logs and scratch files
</commit_message>
<xml_diff>
--- a/docs/Nearz_E2E_Journey_Suite.xlsx
+++ b/docs/Nearz_E2E_Journey_Suite.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -91,6 +91,9 @@
       <family val="0"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -171,7 +174,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -341,6 +344,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7213,7 +7217,7 @@
       </c>
       <c r="B127" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C127" s="43" t="n"/>
@@ -7262,7 +7266,7 @@
       </c>
       <c r="B128" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C128" s="43" t="n"/>
@@ -7311,7 +7315,7 @@
       </c>
       <c r="B129" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C129" s="43" t="n"/>
@@ -7360,7 +7364,7 @@
       </c>
       <c r="B130" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C130" s="43" t="n"/>
@@ -7409,7 +7413,7 @@
       </c>
       <c r="B131" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C131" s="43" t="n"/>
@@ -7458,7 +7462,7 @@
       </c>
       <c r="B132" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C132" s="43" t="n"/>
@@ -7507,7 +7511,7 @@
       </c>
       <c r="B133" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C133" s="43" t="n"/>
@@ -7556,7 +7560,7 @@
       </c>
       <c r="B134" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C134" s="43" t="n"/>
@@ -7605,7 +7609,7 @@
       </c>
       <c r="B135" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C135" s="43" t="n"/>
@@ -7654,7 +7658,7 @@
       </c>
       <c r="B136" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C136" s="43" t="n"/>
@@ -7703,7 +7707,7 @@
       </c>
       <c r="B137" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C137" s="43" t="n"/>
@@ -7752,10 +7756,14 @@
       </c>
       <c r="B138" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C138" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C138" s="43" t="inlineStr">
+        <is>
+          <t>Finding A: the staff ROW splits service/product revenue correctly, the summary CARD does not</t>
+        </is>
+      </c>
       <c r="D138" s="44" t="inlineStr">
         <is>
           <t>6</t>
@@ -7801,7 +7809,7 @@
       </c>
       <c r="B139" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C139" s="43" t="n"/>
@@ -7850,7 +7858,7 @@
       </c>
       <c r="B140" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C140" s="43" t="n"/>
@@ -7899,7 +7907,7 @@
       </c>
       <c r="B141" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C141" s="43" t="n"/>
@@ -7948,7 +7956,7 @@
       </c>
       <c r="B142" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C142" s="43" t="n"/>
@@ -7997,7 +8005,7 @@
       </c>
       <c r="B143" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C143" s="43" t="n"/>
@@ -8046,7 +8054,7 @@
       </c>
       <c r="B144" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C144" s="43" t="n"/>
@@ -8095,7 +8103,7 @@
       </c>
       <c r="B145" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C145" s="43" t="n"/>
@@ -8144,7 +8152,7 @@
       </c>
       <c r="B146" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C146" s="43" t="n"/>
@@ -8193,7 +8201,7 @@
       </c>
       <c r="B147" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C147" s="43" t="n"/>
@@ -8242,7 +8250,7 @@
       </c>
       <c r="B148" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C148" s="43" t="n"/>
@@ -8291,7 +8299,7 @@
       </c>
       <c r="B149" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C149" s="43" t="n"/>
@@ -8340,10 +8348,14 @@
       </c>
       <c r="B150" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C150" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C150" s="43" t="inlineStr">
+        <is>
+          <t>D18 is asserted separately in Block 4; this case covers assignment changes only</t>
+        </is>
+      </c>
       <c r="D150" s="44" t="inlineStr">
         <is>
           <t>6</t>
@@ -8389,7 +8401,7 @@
       </c>
       <c r="B151" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C151" s="43" t="n"/>
@@ -8438,7 +8450,7 @@
       </c>
       <c r="B152" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C152" s="43" t="n"/>
@@ -8487,7 +8499,7 @@
       </c>
       <c r="B153" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C153" s="43" t="n"/>
@@ -8536,7 +8548,7 @@
       </c>
       <c r="B154" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C154" s="43" t="n"/>
@@ -8585,7 +8597,7 @@
       </c>
       <c r="B155" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C155" s="43" t="n"/>
@@ -8634,7 +8646,7 @@
       </c>
       <c r="B156" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C156" s="43" t="n"/>
@@ -8683,7 +8695,7 @@
       </c>
       <c r="B157" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C157" s="43" t="n"/>
@@ -8732,10 +8744,14 @@
       </c>
       <c r="B158" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C158" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C158" s="43" t="inlineStr">
+        <is>
+          <t>part refund issues a credit note (CN-NRZ-...) carrying its own CGST/SGST split</t>
+        </is>
+      </c>
       <c r="D158" s="44" t="inlineStr">
         <is>
           <t>7</t>
@@ -8781,7 +8797,7 @@
       </c>
       <c r="B159" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C159" s="43" t="n"/>
@@ -8830,7 +8846,7 @@
       </c>
       <c r="B160" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C160" s="43" t="n"/>
@@ -8879,7 +8895,7 @@
       </c>
       <c r="B161" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C161" s="43" t="n"/>
@@ -8928,7 +8944,7 @@
       </c>
       <c r="B162" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C162" s="43" t="n"/>
@@ -8977,7 +8993,7 @@
       </c>
       <c r="B163" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C163" s="43" t="n"/>
@@ -9026,7 +9042,7 @@
       </c>
       <c r="B164" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C164" s="43" t="n"/>
@@ -9075,7 +9091,7 @@
       </c>
       <c r="B165" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C165" s="43" t="n"/>
@@ -9124,7 +9140,7 @@
       </c>
       <c r="B166" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C166" s="43" t="n"/>
@@ -9173,10 +9189,14 @@
       </c>
       <c r="B167" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C167" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C167" s="43" t="inlineStr">
+        <is>
+          <t>zero stock: the DRAFT is accepted, the SETTLE is refused 422 "Insufficient stock"</t>
+        </is>
+      </c>
       <c r="D167" s="44" t="inlineStr">
         <is>
           <t>7</t>
@@ -9222,10 +9242,14 @@
       </c>
       <c r="B168" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C168" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C168" s="43" t="inlineStr">
+        <is>
+          <t>was parked a few hours on 7 Sep - the write route is POST /expenses, not /salons/{id}/expenses; unparked same day</t>
+        </is>
+      </c>
       <c r="D168" s="44" t="inlineStr">
         <is>
           <t>7</t>
@@ -9271,10 +9295,14 @@
       </c>
       <c r="B169" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C169" s="43" t="n"/>
+          <t>BUILT - failing (known-defect)</t>
+        </is>
+      </c>
+      <c r="C169" s="43" t="inlineStr">
+        <is>
+          <t>D19: a full refund returns the revenue AND the stock but keeps COGS booked, so profit is short by the cost price</t>
+        </is>
+      </c>
       <c r="D169" s="44" t="inlineStr">
         <is>
           <t>7</t>
@@ -9320,7 +9348,7 @@
       </c>
       <c r="B170" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C170" s="43" t="n"/>
@@ -9369,7 +9397,7 @@
       </c>
       <c r="B171" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C171" s="43" t="n"/>
@@ -9418,7 +9446,7 @@
       </c>
       <c r="B172" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C172" s="43" t="n"/>
@@ -9467,7 +9495,7 @@
       </c>
       <c r="B173" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C173" s="43" t="n"/>
@@ -9516,7 +9544,7 @@
       </c>
       <c r="B174" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C174" s="43" t="n"/>
@@ -9565,7 +9593,7 @@
       </c>
       <c r="B175" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C175" s="43" t="n"/>
@@ -9614,10 +9642,14 @@
       </c>
       <c r="B176" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C176" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C176" s="43" t="inlineStr">
+        <is>
+          <t>holds the line on Credit vs Debit - salon 4550 carries 160,000 of auto-written Credit rows that must never count as cost</t>
+        </is>
+      </c>
       <c r="D176" s="44" t="inlineStr">
         <is>
           <t>8</t>
@@ -9663,10 +9695,14 @@
       </c>
       <c r="B177" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C177" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C177" s="43" t="inlineStr">
+        <is>
+          <t>backdated expense stays in the past - the range boundary from the cost side</t>
+        </is>
+      </c>
       <c r="D177" s="44" t="inlineStr">
         <is>
           <t>8</t>
@@ -9712,7 +9748,7 @@
       </c>
       <c r="B178" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C178" s="43" t="n"/>
@@ -9761,7 +9797,7 @@
       </c>
       <c r="B179" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C179" s="43" t="n"/>
@@ -9810,10 +9846,14 @@
       </c>
       <c r="B180" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C180" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C180" s="43" t="inlineStr">
+        <is>
+          <t>the dashboard panel keeps its total at data.summary.total.value; its "recent" list is NOT range-filtered</t>
+        </is>
+      </c>
       <c r="D180" s="44" t="inlineStr">
         <is>
           <t>8</t>
@@ -9859,7 +9899,7 @@
       </c>
       <c r="B181" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C181" s="43" t="n"/>
@@ -9908,7 +9948,7 @@
       </c>
       <c r="B182" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C182" s="43" t="n"/>
@@ -9957,10 +9997,14 @@
       </c>
       <c r="B183" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C183" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C183" s="43" t="inlineStr">
+        <is>
+          <t>a product taken to its reorder level must appear on the dashboard low-stock list</t>
+        </is>
+      </c>
       <c r="D183" s="44" t="inlineStr">
         <is>
           <t>9</t>
@@ -10006,7 +10050,7 @@
       </c>
       <c r="B184" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C184" s="43" t="n"/>
@@ -10055,7 +10099,7 @@
       </c>
       <c r="B185" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C185" s="43" t="n"/>
@@ -10104,10 +10148,14 @@
       </c>
       <c r="B186" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C186" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C186" s="43" t="inlineStr">
+        <is>
+          <t>asserts ABSOLUTE equality between dashboard and reports, not just matching deltas</t>
+        </is>
+      </c>
       <c r="D186" s="44" t="inlineStr">
         <is>
           <t>9</t>
@@ -10153,7 +10201,7 @@
       </c>
       <c r="B187" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C187" s="43" t="n"/>
@@ -10202,7 +10250,7 @@
       </c>
       <c r="B188" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C188" s="43" t="n"/>
@@ -10251,10 +10299,14 @@
       </c>
       <c r="B189" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C189" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C189" s="43" t="inlineStr">
+        <is>
+          <t>the staff report counts TAX-INCLUSIVE revenue - 1,000 service shows as 1,180 on the row</t>
+        </is>
+      </c>
       <c r="D189" s="44" t="inlineStr">
         <is>
           <t>10</t>
@@ -10300,10 +10352,14 @@
       </c>
       <c r="B190" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C190" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C190" s="43" t="inlineStr">
+        <is>
+          <t>the API answers "Cancelled" with a capital C; assertAppointmentIs normalises it</t>
+        </is>
+      </c>
       <c r="D190" s="44" t="inlineStr">
         <is>
           <t>10</t>
@@ -10349,7 +10405,7 @@
       </c>
       <c r="B191" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C191" s="43" t="n"/>
@@ -10398,7 +10454,7 @@
       </c>
       <c r="B192" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C192" s="43" t="n"/>
@@ -10447,7 +10503,7 @@
       </c>
       <c r="B193" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C193" s="43" t="n"/>
@@ -10496,7 +10552,7 @@
       </c>
       <c r="B194" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C194" s="43" t="n"/>
@@ -10545,7 +10601,7 @@
       </c>
       <c r="B195" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C195" s="43" t="n"/>
@@ -10594,7 +10650,7 @@
       </c>
       <c r="B196" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C196" s="43" t="n"/>
@@ -10643,10 +10699,14 @@
       </c>
       <c r="B197" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C197" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C197" s="43" t="inlineStr">
+        <is>
+          <t>service_cogs deliberately not asserted here - D19 would make one bug fail two tests</t>
+        </is>
+      </c>
       <c r="D197" s="44" t="inlineStr">
         <is>
           <t>10</t>
@@ -10692,7 +10752,7 @@
       </c>
       <c r="B198" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C198" s="43" t="n"/>
@@ -10741,7 +10801,7 @@
       </c>
       <c r="B199" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
+          <t>BUILT - passing</t>
         </is>
       </c>
       <c r="C199" s="43" t="n"/>
@@ -10790,10 +10850,14 @@
       </c>
       <c r="B200" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C200" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C200" s="43" t="inlineStr">
+        <is>
+          <t>standing regression on D17 and D18; goes RED when either is fixed, which is the signal to rewrite it</t>
+        </is>
+      </c>
       <c r="D200" s="44" t="inlineStr">
         <is>
           <t>10</t>
@@ -10839,10 +10903,14 @@
       </c>
       <c r="B201" s="43" t="inlineStr">
         <is>
-          <t>TO WRITE</t>
-        </is>
-      </c>
-      <c r="C201" s="43" t="n"/>
+          <t>BUILT - passing</t>
+        </is>
+      </c>
+      <c r="C201" s="43" t="inlineStr">
+        <is>
+          <t>the closing journey - books, shelf, staff report, dashboard and P&amp;L reconciled at once</t>
+        </is>
+      </c>
       <c r="D201" s="44" t="inlineStr">
         <is>
           <t>10</t>
@@ -11174,13 +11242,13 @@
         <v>25</v>
       </c>
       <c r="E7" s="48" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F7" s="48" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="48" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H7" s="48" t="n">
         <v>239</v>
@@ -11191,7 +11259,7 @@
       </c>
       <c r="J7" s="48" t="inlineStr">
         <is>
-          <t>to write</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -11213,13 +11281,13 @@
         <v>20</v>
       </c>
       <c r="E8" s="48" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F8" s="48" t="n">
         <v>0</v>
       </c>
       <c r="G8" s="48" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H8" s="48" t="n">
         <v>245</v>
@@ -11230,7 +11298,7 @@
       </c>
       <c r="J8" s="48" t="inlineStr">
         <is>
-          <t>to write</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -11252,13 +11320,13 @@
         <v>10</v>
       </c>
       <c r="E9" s="48" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F9" s="48" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="48" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H9" s="48" t="n">
         <v>125</v>
@@ -11269,7 +11337,7 @@
       </c>
       <c r="J9" s="48" t="inlineStr">
         <is>
-          <t>to write</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -11291,13 +11359,13 @@
         <v>5</v>
       </c>
       <c r="E10" s="48" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F10" s="48" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="48" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H10" s="48" t="n">
         <v>47</v>
@@ -11308,7 +11376,7 @@
       </c>
       <c r="J10" s="48" t="inlineStr">
         <is>
-          <t>to write</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -11330,13 +11398,13 @@
         <v>15</v>
       </c>
       <c r="E11" s="48" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F11" s="48" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="48" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H11" s="48" t="n">
         <v>257</v>
@@ -11347,7 +11415,7 @@
       </c>
       <c r="J11" s="48" t="inlineStr">
         <is>
-          <t>to write</t>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -11422,7 +11490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A96"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="100" customWidth="1" style="28" min="1" max="1"/>
@@ -11448,14 +11516,14 @@
     <row r="4" ht="15" customHeight="1" s="29">
       <c r="A4" s="56" t="inlineStr">
         <is>
-          <t>BUILT - passing    56 journeys written, run against the live QA API, green.</t>
+          <t>BUILT - passing   174 journeys written, run against the live QA API, green.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="29">
       <c r="A5" s="56" t="inlineStr">
         <is>
-          <t>PARKED             19 written and skip-marked. 17 need partial payments, which are off</t>
+          <t>PARKED             21 written and skip-marked. 19 need partial payments, which are off</t>
         </is>
       </c>
     </row>
@@ -11469,14 +11537,14 @@
     <row r="7" ht="15" customHeight="1" s="29">
       <c r="A7" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">                   covered by 119. Each is one 'skip=' away from running.</t>
+          <t xml:space="preserve">                   in the frontend; 015 needs the split-payment modes[] payload; 068 is</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="29">
       <c r="A8" s="56" t="inlineStr">
         <is>
-          <t>TO WRITE          125 journeys, blocks 4 to 10.</t>
+          <t>BUILT - failing     2 deliberately failing in the known-defect group: 049 (D18) and</t>
         </is>
       </c>
     </row>
@@ -11580,6 +11648,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="28" t="inlineStr">
         <is>
@@ -11601,6 +11670,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="28" t="inlineStr">
         <is>
@@ -11629,31 +11699,365 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="28" t="inlineStr">
         <is>
           <t>4 Sep 2026 - Block 5 (build order) built: API-E2E-051..075, bill construction</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="28" t="inlineStr">
         <is>
           <t>24 passing, 1 parked (068 - split payment needs partial payment, off in the frontend).</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="28" t="inlineStr">
         <is>
           <t>The automation now lives in Documents\nearz-api-tests. api-service holds no test code at all.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="28" t="inlineStr">
         <is>
           <t>Block 5 corrected the Profit model: gross_revenue is net_payable MINUS tax (so a rounded bill keeps 40p less), and net_profit then deducts cost of goods sold. Both only show up on baskets with a product and a discount - which is why they survived 100 earlier tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="57" t="inlineStr">
+        <is>
+          <t>7 Sep 2026 - blocks 6 to 10 built: the suite is complete at 200 journeys</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="28" t="inlineStr">
+        <is>
+          <t>Block 6  API-E2E-126..150  staff, attendance and commission.  25/25 passing first run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
+          <t>Block 7  API-E2E-151..170  products and inventory.  19 passing, 1 known-defect (168 = D19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="28" t="inlineStr">
+        <is>
+          <t>Block 8  API-E2E-171..180  expenses and profit.  10/10 passing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="28" t="inlineStr">
+        <is>
+          <t>Block 9  API-E2E-181..185  dashboard reconciliation.  5/5 passing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="28" t="inlineStr">
+        <is>
+          <t>Block 10 API-E2E-186..200  composite mega-journeys.  15/15 passing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" s="28" t="inlineStr">
+        <is>
+          <t>Totals: 174 passing, 21 parked, 2 deliberately failing, 3 removed as duplicates = 200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="57" t="inlineStr">
+        <is>
+          <t>Found while building these five blocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="28" t="inlineStr">
+        <is>
+          <t>D19  A full refund gives back the revenue AND the stock but keeps the cost of goods sold</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     booked. The bottle is on the shelf again and its cost will be charged a second time</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     when it sells. Measured: revenue -200 reversed, COGS +100 stayed, net profit -100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     The error compounds - sell and refund one bottle ten times and the books carry 1,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     of cost for goods that never left the building.  Pinned by e2e168 (known-defect).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="28" t="inlineStr">
+        <is>
+          <t>D1   Narrowed. The 4 Sep re-verification said "not reproduced" after checking bills and</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     appointments. Too broad: staffs#show and products#show still answer HTTP 200 with</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     {"error":"not_found"} - and products#show does it for a product that EXISTS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="28" t="inlineStr">
+        <is>
+          <t>F    The expense WRITE route is POST /expenses, not POST /salons/{id}/expenses (404).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     The salon comes from the token, so you cannot write an expense for a salon you can read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="28" t="inlineStr">
+        <is>
+          <t>G    Every completed appointment auto-writes a CREDIT expense row for the service price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Salon 4550 carries 160,000 of them. Operating Expenses correctly excludes Credit rows -</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     e2e175 exists to keep it that way, because if that filter were ever dropped this salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     would appear to have spent its entire revenue on nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65"/>
+    <row r="66">
+      <c r="A66" s="57" t="inlineStr">
+        <is>
+          <t>Corrections made to the tests themselves (the API was right)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="28" t="inlineStr">
+        <is>
+          <t>The Staff Performance report counts TAX-INCLUSIVE revenue: a 1,000 service on an 18% salon</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="28" t="inlineStr">
+        <is>
+          <t>shows as 1,180 on the stylist row. Block 10 was written against the ex-tax figure and six</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="28" t="inlineStr">
+        <is>
+          <t>tests failed until it was fixed. Block 6 already had this right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="28" t="inlineStr">
+        <is>
+          <t>payment_summary on the dashboard is a LIST of payment modes, not one object - it only looks</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="28" t="inlineStr">
+        <is>
+          <t>like an object on a day with a single mode. Now summed, which also proves the split adds up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73"/>
+    <row r="74">
+      <c r="A74" s="57" t="inlineStr">
+        <is>
+          <t>7 Sep 2026 - first full-suite run: read this before running all 200 at once</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Result: 201 run, 146 passed, 21 skipped by design, 34 failed - and ZERO of the 34 was an</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>assertion. Every one was the same IllegalState:</t>
+        </is>
+      </c>
+    </row>
+    <row r="77"/>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    today's calendar is full: all 380 places (19 slots x 20 stylists) are taken</t>
+        </is>
+      </c>
+    </row>
+    <row r="79"/>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Not a defect and not a test bug. Appointment slots are a budget PER DAY, not per run -</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>an appointment booked at 11am still occupies its slot at 6pm. Each of the ten blocks had</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>already been run individually the same day (several of them twice, after a fix), and the</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>salon was carrying ~94 appointments before the full run even started. The suite ran out of</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>calendar partway through Block 2 and everything after it inherited the same failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85"/>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Two ways to run all 200 in one go:</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. Run it FIRST on a fresh day, before any single-block runs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. Raise ROSTER in Catalogue.java (line 39). Each extra stylist adds 19 slots/day;</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     20 -&gt; 40 gives 760. Catalogue seeds any missing "QA Stylist N" on the next run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90"/>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Budget the day before running: roughly 250 slots, because some journeys book more than</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>one appointment - e2e198 books ten, e2e195 five, e2e192 and e2e197 three each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93"/>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>The 146 that ran is the meaningful number: every arithmetic and report-delta assertion</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>that executed, passed. Each block was also run on its own the same day and was green -</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Block 6 25/25, Block 7 19/19, Block 8 10/10, Block 9 5/5, Block 10 15/15.</t>
         </is>
       </c>
     </row>

</xml_diff>